<commit_message>
round 2 report. Was able to run all the code. Some discrepancies. ReadMe is more complete.
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="67">
   <si>
     <t xml:space="preserve">Data Preparation Program</t>
   </si>
@@ -46,16 +46,61 @@
     <t xml:space="preserve">X_estimate_fe.R</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes, differences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_event_study.do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selection_based_NAM.do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_fixed_effects.do</t>
+  </si>
+  <si>
     <t xml:space="preserve">?</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X_fixed_effects.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, differences</t>
+    <t xml:space="preserve">Figure 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_summary_stats.do</t>
   </si>
   <si>
     <t xml:space="preserve">Figure A.2 </t>
@@ -67,148 +112,115 @@
     <t xml:space="preserve">Figure A.4</t>
   </si>
   <si>
+    <t xml:space="preserve">Table B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B_gender_moves.do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure C1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Figure C.2 </t>
   </si>
   <si>
+    <t xml:space="preserve">Figure C.3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table D1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure D1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure D2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure D.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">simulate_selection.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure E.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_grouped_fixed_effects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure E.2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure E.3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_counterfactuals.do</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes, differences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure G6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In-text numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 52 </t>
+  </si>
+  <si>
     <t xml:space="preserve">no</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure C.3 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure E.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X_grouped_fixed_effects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure E.2 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure E.3 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 5 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">X_event_study.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure A.5 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X_summary_stats.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table D1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X_counterfactuals.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table B2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B_gender_moves.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">selection_based_NAM.do</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure D.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">simulate_selection.py</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Figure G6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In-text numbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Footnote 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discussion in section 3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“Correlated Measurement Error” section on Appendix E.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“numbers cited in the related discussion in the text Figure 7 and Figure A.5”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discussion in Appendix C.1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analysis reported in Appendix F</t>
+    <t xml:space="preserve">p. 72 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes, wrong label in do.file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 73</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p. 10</t>
   </si>
 </sst>
 </file>
@@ -502,8 +514,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D62"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.91"/>
@@ -544,6 +556,10 @@
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
     </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>3</v>
@@ -565,11 +581,11 @@
       <c r="B11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D11" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -577,73 +593,73 @@
         <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>11</v>
+      <c r="D13" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="0" t="s">
-        <v>16</v>
+      <c r="D16" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="0" t="s">
-        <v>16</v>
+      <c r="D17" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -651,10 +667,10 @@
         <v>21</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -662,10 +678,10 @@
         <v>22</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -675,8 +691,8 @@
       <c r="B21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>16</v>
+      <c r="D21" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -684,21 +700,21 @@
         <v>24</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="0" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>11</v>
+      <c r="D23" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -706,10 +722,10 @@
         <v>27</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="0" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -717,10 +733,10 @@
         <v>28</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="0" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -728,322 +744,362 @@
         <v>29</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>20</v>
+        <v>26</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>16</v>
+        <v>33</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D33" s="0" t="s">
-        <v>20</v>
+        <v>26</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D34" s="0" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>16</v>
+        <v>42</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="0" t="s">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="0" t="s">
-        <v>16</v>
+        <v>44</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D40" s="0" t="s">
-        <v>16</v>
+        <v>48</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D41" s="0" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D42" s="0" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D44" s="0" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D45" s="0" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D46" s="0" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
+      <c r="A47" s="0"/>
+      <c r="B47" s="0"/>
+      <c r="C47" s="0"/>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0"/>
+      <c r="B48" s="0"/>
+      <c r="C48" s="0"/>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0"/>
+      <c r="B49" s="0"/>
+      <c r="C49" s="0"/>
+    </row>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0"/>
+      <c r="B50" s="0"/>
+      <c r="C50" s="0"/>
+    </row>
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0"/>
+      <c r="B51" s="0"/>
+      <c r="C51" s="0"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0"/>
+      <c r="B52" s="0"/>
+      <c r="C52" s="0"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B54" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D49" s="3" t="s">
+      <c r="D54" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="s">
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B55" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D50" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D53" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D54" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D55" s="0" t="s">
-        <v>8</v>
+      <c r="D61" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" s="0" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>